<commit_message>
Desarrollo de cartas de contenidos
</commit_message>
<xml_diff>
--- a/public/templates/cs12.xlsx
+++ b/public/templates/cs12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\saat\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F61D4B03-37B6-45E0-B6B2-EFD7370260E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2076CD78-7637-44C6-B67F-A9F22D9FAD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Central" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="40">
   <si>
     <t>Nº</t>
   </si>
@@ -69,9 +69,6 @@
     <t>(CONSEJEROS Y DIRECCIONES TÉCNICAS)</t>
   </si>
   <si>
-    <t>Grammar</t>
-  </si>
-  <si>
     <t>PROMEDIOS MATERIAS</t>
   </si>
   <si>
@@ -88,9 +85,6 @@
   </si>
   <si>
     <t>Lenguaje</t>
-  </si>
-  <si>
-    <t>Literature</t>
   </si>
   <si>
     <t>P. Inglés</t>
@@ -138,12 +132,6 @@
     <t>PF</t>
   </si>
   <si>
-    <t>Física</t>
-  </si>
-  <si>
-    <t>Química</t>
-  </si>
-  <si>
     <t>CENTRALIZADOR DE NOTAS</t>
   </si>
   <si>
@@ -154,6 +142,21 @@
   </si>
   <si>
     <t>1 de 2</t>
+  </si>
+  <si>
+    <t>Literature [50%]</t>
+  </si>
+  <si>
+    <t>Grammar [50%]</t>
+  </si>
+  <si>
+    <t>Física [10%]</t>
+  </si>
+  <si>
+    <t>C. Naturales [80%]</t>
+  </si>
+  <si>
+    <t>Química [10%]</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1274,23 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1283,26 +1302,23 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1328,37 +1344,24 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="71">
     <cellStyle name="20% - Accent1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1572,7 +1575,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>51</xdr:col>
-      <xdr:colOff>912301</xdr:colOff>
+      <xdr:colOff>756437</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
@@ -1967,717 +1970,717 @@
     <col min="1" max="1" width="3.140625" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="50" width="3.85546875" customWidth="1"/>
-    <col min="51" max="51" width="3" customWidth="1"/>
-    <col min="52" max="52" width="35" customWidth="1"/>
+    <col min="51" max="51" width="5.140625" customWidth="1"/>
+    <col min="52" max="52" width="42.28515625" customWidth="1"/>
     <col min="53" max="64" width="5" customWidth="1"/>
     <col min="65" max="80" width="4.5703125" customWidth="1"/>
     <col min="81" max="82" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="Q2" s="58"/>
-      <c r="R2" s="58"/>
-      <c r="S2" s="58"/>
-      <c r="T2" s="58"/>
-      <c r="U2" s="58"/>
-      <c r="V2" s="58"/>
-      <c r="W2" s="58"/>
-      <c r="X2" s="58"/>
-      <c r="Y2" s="58"/>
-      <c r="Z2" s="58"/>
-      <c r="AA2" s="58"/>
-      <c r="AB2" s="58"/>
-      <c r="AC2" s="58"/>
-      <c r="AD2" s="58"/>
-      <c r="AE2" s="58"/>
-      <c r="AF2" s="58"/>
-      <c r="AG2" s="58"/>
-      <c r="AH2" s="58"/>
-      <c r="AI2" s="58"/>
-      <c r="AJ2" s="58"/>
-      <c r="AK2" s="58"/>
-      <c r="AL2" s="58"/>
-      <c r="AM2" s="58"/>
-      <c r="AN2" s="58"/>
-      <c r="AO2" s="58"/>
-      <c r="AP2" s="58"/>
-      <c r="AQ2" s="58"/>
-      <c r="AR2" s="58"/>
-      <c r="AS2" s="58"/>
-      <c r="AT2" s="58"/>
-      <c r="AU2" s="58"/>
-      <c r="AV2" s="58"/>
-      <c r="AW2" s="58"/>
-      <c r="AX2" s="58"/>
-      <c r="AY2" s="58" t="str">
+      <c r="A2" s="56" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="56"/>
+      <c r="Q2" s="56"/>
+      <c r="R2" s="56"/>
+      <c r="S2" s="56"/>
+      <c r="T2" s="56"/>
+      <c r="U2" s="56"/>
+      <c r="V2" s="56"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="56"/>
+      <c r="Y2" s="56"/>
+      <c r="Z2" s="56"/>
+      <c r="AA2" s="56"/>
+      <c r="AB2" s="56"/>
+      <c r="AC2" s="56"/>
+      <c r="AD2" s="56"/>
+      <c r="AE2" s="56"/>
+      <c r="AF2" s="56"/>
+      <c r="AG2" s="56"/>
+      <c r="AH2" s="56"/>
+      <c r="AI2" s="56"/>
+      <c r="AJ2" s="56"/>
+      <c r="AK2" s="56"/>
+      <c r="AL2" s="56"/>
+      <c r="AM2" s="56"/>
+      <c r="AN2" s="56"/>
+      <c r="AO2" s="56"/>
+      <c r="AP2" s="56"/>
+      <c r="AQ2" s="56"/>
+      <c r="AR2" s="56"/>
+      <c r="AS2" s="56"/>
+      <c r="AT2" s="56"/>
+      <c r="AU2" s="56"/>
+      <c r="AV2" s="56"/>
+      <c r="AW2" s="56"/>
+      <c r="AX2" s="56"/>
+      <c r="AY2" s="56" t="str">
         <f>A2</f>
         <v>CENTRALIZADOR DE NOTAS</v>
       </c>
-      <c r="AZ2" s="58"/>
-      <c r="BA2" s="58"/>
-      <c r="BB2" s="58"/>
-      <c r="BC2" s="58"/>
-      <c r="BD2" s="58"/>
-      <c r="BE2" s="58"/>
-      <c r="BF2" s="58"/>
-      <c r="BG2" s="58"/>
-      <c r="BH2" s="58"/>
-      <c r="BI2" s="58"/>
-      <c r="BJ2" s="58"/>
-      <c r="BK2" s="58"/>
-      <c r="BL2" s="58"/>
-      <c r="BM2" s="58"/>
-      <c r="BN2" s="58"/>
-      <c r="BO2" s="58"/>
-      <c r="BP2" s="58"/>
-      <c r="BQ2" s="58"/>
-      <c r="BR2" s="58"/>
-      <c r="BS2" s="58"/>
-      <c r="BT2" s="58"/>
-      <c r="BU2" s="58"/>
-      <c r="BV2" s="58"/>
-      <c r="BW2" s="58"/>
-      <c r="BX2" s="58"/>
-      <c r="BY2" s="58"/>
-      <c r="BZ2" s="58"/>
-      <c r="CA2" s="58"/>
-      <c r="CB2" s="58"/>
+      <c r="AZ2" s="56"/>
+      <c r="BA2" s="56"/>
+      <c r="BB2" s="56"/>
+      <c r="BC2" s="56"/>
+      <c r="BD2" s="56"/>
+      <c r="BE2" s="56"/>
+      <c r="BF2" s="56"/>
+      <c r="BG2" s="56"/>
+      <c r="BH2" s="56"/>
+      <c r="BI2" s="56"/>
+      <c r="BJ2" s="56"/>
+      <c r="BK2" s="56"/>
+      <c r="BL2" s="56"/>
+      <c r="BM2" s="56"/>
+      <c r="BN2" s="56"/>
+      <c r="BO2" s="56"/>
+      <c r="BP2" s="56"/>
+      <c r="BQ2" s="56"/>
+      <c r="BR2" s="56"/>
+      <c r="BS2" s="56"/>
+      <c r="BT2" s="56"/>
+      <c r="BU2" s="56"/>
+      <c r="BV2" s="56"/>
+      <c r="BW2" s="56"/>
+      <c r="BX2" s="56"/>
+      <c r="BY2" s="56"/>
+      <c r="BZ2" s="56"/>
+      <c r="CA2" s="56"/>
+      <c r="CB2" s="56"/>
     </row>
     <row r="3" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="72"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
-      <c r="I3" s="72"/>
-      <c r="J3" s="72"/>
-      <c r="K3" s="72"/>
-      <c r="L3" s="72"/>
-      <c r="M3" s="72"/>
-      <c r="N3" s="72"/>
-      <c r="O3" s="72"/>
-      <c r="P3" s="72"/>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="72"/>
-      <c r="S3" s="72"/>
-      <c r="T3" s="72"/>
-      <c r="U3" s="72"/>
-      <c r="V3" s="72"/>
-      <c r="W3" s="72"/>
-      <c r="X3" s="72"/>
-      <c r="Y3" s="72"/>
-      <c r="Z3" s="72"/>
-      <c r="AA3" s="72"/>
-      <c r="AB3" s="72"/>
-      <c r="AC3" s="72"/>
-      <c r="AD3" s="72"/>
-      <c r="AE3" s="72"/>
-      <c r="AF3" s="72"/>
-      <c r="AG3" s="72"/>
-      <c r="AH3" s="72"/>
-      <c r="AI3" s="72"/>
-      <c r="AJ3" s="72"/>
-      <c r="AK3" s="72"/>
-      <c r="AL3" s="72"/>
-      <c r="AM3" s="72"/>
-      <c r="AN3" s="72"/>
-      <c r="AO3" s="72"/>
-      <c r="AP3" s="72"/>
-      <c r="AQ3" s="72"/>
-      <c r="AR3" s="72"/>
-      <c r="AS3" s="72"/>
-      <c r="AT3" s="72"/>
-      <c r="AU3" s="72"/>
-      <c r="AV3" s="72"/>
-      <c r="AW3" s="72"/>
-      <c r="AX3" s="72"/>
-      <c r="AY3" s="58" t="str">
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="57"/>
+      <c r="W3" s="57"/>
+      <c r="X3" s="57"/>
+      <c r="Y3" s="57"/>
+      <c r="Z3" s="57"/>
+      <c r="AA3" s="57"/>
+      <c r="AB3" s="57"/>
+      <c r="AC3" s="57"/>
+      <c r="AD3" s="57"/>
+      <c r="AE3" s="57"/>
+      <c r="AF3" s="57"/>
+      <c r="AG3" s="57"/>
+      <c r="AH3" s="57"/>
+      <c r="AI3" s="57"/>
+      <c r="AJ3" s="57"/>
+      <c r="AK3" s="57"/>
+      <c r="AL3" s="57"/>
+      <c r="AM3" s="57"/>
+      <c r="AN3" s="57"/>
+      <c r="AO3" s="57"/>
+      <c r="AP3" s="57"/>
+      <c r="AQ3" s="57"/>
+      <c r="AR3" s="57"/>
+      <c r="AS3" s="57"/>
+      <c r="AT3" s="57"/>
+      <c r="AU3" s="57"/>
+      <c r="AV3" s="57"/>
+      <c r="AW3" s="57"/>
+      <c r="AX3" s="57"/>
+      <c r="AY3" s="56" t="str">
         <f t="shared" ref="AY3:AY4" si="0">A3</f>
         <v>(CONSEJEROS Y DIRECCIONES TÉCNICAS)</v>
       </c>
-      <c r="AZ3" s="58"/>
-      <c r="BA3" s="58"/>
-      <c r="BB3" s="58"/>
-      <c r="BC3" s="58"/>
-      <c r="BD3" s="58"/>
-      <c r="BE3" s="58"/>
-      <c r="BF3" s="58"/>
-      <c r="BG3" s="58"/>
-      <c r="BH3" s="58"/>
-      <c r="BI3" s="58"/>
-      <c r="BJ3" s="58"/>
-      <c r="BK3" s="58"/>
-      <c r="BL3" s="58"/>
-      <c r="BM3" s="58"/>
-      <c r="BN3" s="58"/>
-      <c r="BO3" s="58"/>
-      <c r="BP3" s="58"/>
-      <c r="BQ3" s="58"/>
-      <c r="BR3" s="58"/>
-      <c r="BS3" s="58"/>
-      <c r="BT3" s="58"/>
-      <c r="BU3" s="58"/>
-      <c r="BV3" s="58"/>
-      <c r="BW3" s="58"/>
-      <c r="BX3" s="58"/>
-      <c r="BY3" s="58"/>
-      <c r="BZ3" s="58"/>
-      <c r="CA3" s="58"/>
-      <c r="CB3" s="58"/>
+      <c r="AZ3" s="56"/>
+      <c r="BA3" s="56"/>
+      <c r="BB3" s="56"/>
+      <c r="BC3" s="56"/>
+      <c r="BD3" s="56"/>
+      <c r="BE3" s="56"/>
+      <c r="BF3" s="56"/>
+      <c r="BG3" s="56"/>
+      <c r="BH3" s="56"/>
+      <c r="BI3" s="56"/>
+      <c r="BJ3" s="56"/>
+      <c r="BK3" s="56"/>
+      <c r="BL3" s="56"/>
+      <c r="BM3" s="56"/>
+      <c r="BN3" s="56"/>
+      <c r="BO3" s="56"/>
+      <c r="BP3" s="56"/>
+      <c r="BQ3" s="56"/>
+      <c r="BR3" s="56"/>
+      <c r="BS3" s="56"/>
+      <c r="BT3" s="56"/>
+      <c r="BU3" s="56"/>
+      <c r="BV3" s="56"/>
+      <c r="BW3" s="56"/>
+      <c r="BX3" s="56"/>
+      <c r="BY3" s="56"/>
+      <c r="BZ3" s="56"/>
+      <c r="CA3" s="56"/>
+      <c r="CB3" s="56"/>
     </row>
     <row r="4" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A4" s="73"/>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
-      <c r="N4" s="73"/>
-      <c r="O4" s="73"/>
-      <c r="P4" s="73"/>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-      <c r="S4" s="73"/>
-      <c r="T4" s="73"/>
-      <c r="U4" s="73"/>
-      <c r="V4" s="73"/>
-      <c r="W4" s="73"/>
-      <c r="X4" s="73"/>
-      <c r="Y4" s="73"/>
-      <c r="Z4" s="73"/>
-      <c r="AA4" s="73"/>
-      <c r="AB4" s="73"/>
-      <c r="AC4" s="73"/>
-      <c r="AD4" s="73"/>
-      <c r="AE4" s="73"/>
-      <c r="AF4" s="73"/>
-      <c r="AG4" s="73"/>
-      <c r="AH4" s="73"/>
-      <c r="AI4" s="73"/>
-      <c r="AJ4" s="73"/>
-      <c r="AK4" s="73"/>
-      <c r="AL4" s="73"/>
-      <c r="AM4" s="73"/>
-      <c r="AN4" s="73"/>
-      <c r="AO4" s="73"/>
-      <c r="AP4" s="73"/>
-      <c r="AQ4" s="73"/>
-      <c r="AR4" s="73"/>
-      <c r="AS4" s="73"/>
-      <c r="AT4" s="73"/>
-      <c r="AU4" s="73"/>
-      <c r="AV4" s="73"/>
-      <c r="AW4" s="73"/>
-      <c r="AX4" s="73"/>
-      <c r="AY4" s="58">
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
+      <c r="V4" s="58"/>
+      <c r="W4" s="58"/>
+      <c r="X4" s="58"/>
+      <c r="Y4" s="58"/>
+      <c r="Z4" s="58"/>
+      <c r="AA4" s="58"/>
+      <c r="AB4" s="58"/>
+      <c r="AC4" s="58"/>
+      <c r="AD4" s="58"/>
+      <c r="AE4" s="58"/>
+      <c r="AF4" s="58"/>
+      <c r="AG4" s="58"/>
+      <c r="AH4" s="58"/>
+      <c r="AI4" s="58"/>
+      <c r="AJ4" s="58"/>
+      <c r="AK4" s="58"/>
+      <c r="AL4" s="58"/>
+      <c r="AM4" s="58"/>
+      <c r="AN4" s="58"/>
+      <c r="AO4" s="58"/>
+      <c r="AP4" s="58"/>
+      <c r="AQ4" s="58"/>
+      <c r="AR4" s="58"/>
+      <c r="AS4" s="58"/>
+      <c r="AT4" s="58"/>
+      <c r="AU4" s="58"/>
+      <c r="AV4" s="58"/>
+      <c r="AW4" s="58"/>
+      <c r="AX4" s="58"/>
+      <c r="AY4" s="56">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="AZ4" s="58"/>
-      <c r="BA4" s="58"/>
-      <c r="BB4" s="58"/>
-      <c r="BC4" s="58"/>
-      <c r="BD4" s="58"/>
-      <c r="BE4" s="58"/>
-      <c r="BF4" s="58"/>
-      <c r="BG4" s="58"/>
-      <c r="BH4" s="58"/>
-      <c r="BI4" s="58"/>
-      <c r="BJ4" s="58"/>
-      <c r="BK4" s="58"/>
-      <c r="BL4" s="58"/>
-      <c r="BM4" s="58"/>
-      <c r="BN4" s="58"/>
-      <c r="BO4" s="58"/>
-      <c r="BP4" s="58"/>
-      <c r="BQ4" s="58"/>
-      <c r="BR4" s="58"/>
-      <c r="BS4" s="58"/>
-      <c r="BT4" s="58"/>
-      <c r="BU4" s="58"/>
-      <c r="BV4" s="58"/>
-      <c r="BW4" s="58"/>
-      <c r="BX4" s="58"/>
-      <c r="BY4" s="58"/>
-      <c r="BZ4" s="58"/>
-      <c r="CA4" s="58"/>
-      <c r="CB4" s="58"/>
+      <c r="AZ4" s="56"/>
+      <c r="BA4" s="56"/>
+      <c r="BB4" s="56"/>
+      <c r="BC4" s="56"/>
+      <c r="BD4" s="56"/>
+      <c r="BE4" s="56"/>
+      <c r="BF4" s="56"/>
+      <c r="BG4" s="56"/>
+      <c r="BH4" s="56"/>
+      <c r="BI4" s="56"/>
+      <c r="BJ4" s="56"/>
+      <c r="BK4" s="56"/>
+      <c r="BL4" s="56"/>
+      <c r="BM4" s="56"/>
+      <c r="BN4" s="56"/>
+      <c r="BO4" s="56"/>
+      <c r="BP4" s="56"/>
+      <c r="BQ4" s="56"/>
+      <c r="BR4" s="56"/>
+      <c r="BS4" s="56"/>
+      <c r="BT4" s="56"/>
+      <c r="BU4" s="56"/>
+      <c r="BV4" s="56"/>
+      <c r="BW4" s="56"/>
+      <c r="BX4" s="56"/>
+      <c r="BY4" s="56"/>
+      <c r="BZ4" s="56"/>
+      <c r="CA4" s="56"/>
+      <c r="CB4" s="56"/>
     </row>
     <row r="5" spans="1:80" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="74"/>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="74"/>
-      <c r="J5" s="74"/>
-      <c r="K5" s="74"/>
-      <c r="L5" s="74"/>
-      <c r="M5" s="74"/>
-      <c r="N5" s="74"/>
-      <c r="O5" s="74"/>
-      <c r="P5" s="74"/>
-      <c r="Q5" s="74"/>
-      <c r="R5" s="74"/>
-      <c r="S5" s="74"/>
-      <c r="T5" s="74"/>
-      <c r="U5" s="74"/>
-      <c r="V5" s="74"/>
-      <c r="W5" s="74"/>
-      <c r="X5" s="74"/>
-      <c r="Y5" s="74"/>
-      <c r="Z5" s="74"/>
-      <c r="AA5" s="74"/>
-      <c r="AB5" s="74"/>
-      <c r="AC5" s="74"/>
-      <c r="AD5" s="74"/>
-      <c r="AE5" s="74"/>
-      <c r="AF5" s="74"/>
-      <c r="AG5" s="74"/>
-      <c r="AH5" s="74"/>
-      <c r="AI5" s="74"/>
-      <c r="AJ5" s="74"/>
-      <c r="AK5" s="74"/>
-      <c r="AL5" s="74"/>
-      <c r="AM5" s="74"/>
-      <c r="AN5" s="74"/>
-      <c r="AO5" s="74"/>
-      <c r="AP5" s="74"/>
-      <c r="AQ5" s="74"/>
-      <c r="AR5" s="74"/>
-      <c r="AS5" s="74"/>
-      <c r="AT5" s="74"/>
-      <c r="AU5" s="74"/>
-      <c r="AV5" s="74"/>
-      <c r="AW5" s="74"/>
-      <c r="AX5" s="74"/>
-      <c r="AY5" s="59">
+      <c r="A5" s="59"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="59"/>
+      <c r="L5" s="59"/>
+      <c r="M5" s="59"/>
+      <c r="N5" s="59"/>
+      <c r="O5" s="59"/>
+      <c r="P5" s="59"/>
+      <c r="Q5" s="59"/>
+      <c r="R5" s="59"/>
+      <c r="S5" s="59"/>
+      <c r="T5" s="59"/>
+      <c r="U5" s="59"/>
+      <c r="V5" s="59"/>
+      <c r="W5" s="59"/>
+      <c r="X5" s="59"/>
+      <c r="Y5" s="59"/>
+      <c r="Z5" s="59"/>
+      <c r="AA5" s="59"/>
+      <c r="AB5" s="59"/>
+      <c r="AC5" s="59"/>
+      <c r="AD5" s="59"/>
+      <c r="AE5" s="59"/>
+      <c r="AF5" s="59"/>
+      <c r="AG5" s="59"/>
+      <c r="AH5" s="59"/>
+      <c r="AI5" s="59"/>
+      <c r="AJ5" s="59"/>
+      <c r="AK5" s="59"/>
+      <c r="AL5" s="59"/>
+      <c r="AM5" s="59"/>
+      <c r="AN5" s="59"/>
+      <c r="AO5" s="59"/>
+      <c r="AP5" s="59"/>
+      <c r="AQ5" s="59"/>
+      <c r="AR5" s="59"/>
+      <c r="AS5" s="59"/>
+      <c r="AT5" s="59"/>
+      <c r="AU5" s="59"/>
+      <c r="AV5" s="59"/>
+      <c r="AW5" s="59"/>
+      <c r="AX5" s="59"/>
+      <c r="AY5" s="80">
         <f>A5</f>
         <v>0</v>
       </c>
-      <c r="AZ5" s="59"/>
-      <c r="BA5" s="59"/>
-      <c r="BB5" s="59"/>
-      <c r="BC5" s="59"/>
-      <c r="BD5" s="59"/>
-      <c r="BE5" s="59"/>
-      <c r="BF5" s="59"/>
-      <c r="BG5" s="59"/>
-      <c r="BH5" s="59"/>
-      <c r="BI5" s="59"/>
-      <c r="BJ5" s="59"/>
-      <c r="BK5" s="59"/>
-      <c r="BL5" s="59"/>
-      <c r="BM5" s="59"/>
-      <c r="BN5" s="59"/>
-      <c r="BO5" s="59"/>
-      <c r="BP5" s="59"/>
-      <c r="BQ5" s="59"/>
-      <c r="BR5" s="59"/>
-      <c r="BS5" s="59"/>
-      <c r="BT5" s="59"/>
-      <c r="BU5" s="59"/>
-      <c r="BV5" s="59"/>
-      <c r="BW5" s="59"/>
-      <c r="BX5" s="59"/>
-      <c r="BY5" s="59"/>
-      <c r="BZ5" s="59"/>
-      <c r="CA5" s="59"/>
-      <c r="CB5" s="59"/>
+      <c r="AZ5" s="80"/>
+      <c r="BA5" s="80"/>
+      <c r="BB5" s="80"/>
+      <c r="BC5" s="80"/>
+      <c r="BD5" s="80"/>
+      <c r="BE5" s="80"/>
+      <c r="BF5" s="80"/>
+      <c r="BG5" s="80"/>
+      <c r="BH5" s="80"/>
+      <c r="BI5" s="80"/>
+      <c r="BJ5" s="80"/>
+      <c r="BK5" s="80"/>
+      <c r="BL5" s="80"/>
+      <c r="BM5" s="80"/>
+      <c r="BN5" s="80"/>
+      <c r="BO5" s="80"/>
+      <c r="BP5" s="80"/>
+      <c r="BQ5" s="80"/>
+      <c r="BR5" s="80"/>
+      <c r="BS5" s="80"/>
+      <c r="BT5" s="80"/>
+      <c r="BU5" s="80"/>
+      <c r="BV5" s="80"/>
+      <c r="BW5" s="80"/>
+      <c r="BX5" s="80"/>
+      <c r="BY5" s="80"/>
+      <c r="BZ5" s="80"/>
+      <c r="CA5" s="80"/>
+      <c r="CB5" s="80"/>
     </row>
     <row r="6" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="68" t="s">
+      <c r="B6" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="60" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="61"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="55"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="54" t="s">
+      <c r="H6" s="61"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="60" t="s">
+        <v>2</v>
+      </c>
+      <c r="L6" s="61"/>
+      <c r="M6" s="62"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="60" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" s="61"/>
+      <c r="Q6" s="62"/>
+      <c r="R6" s="64"/>
+      <c r="S6" s="60" t="s">
+        <v>4</v>
+      </c>
+      <c r="T6" s="61"/>
+      <c r="U6" s="62"/>
+      <c r="V6" s="62"/>
+      <c r="W6" s="60" t="s">
+        <v>17</v>
+      </c>
+      <c r="X6" s="61"/>
+      <c r="Y6" s="62"/>
+      <c r="Z6" s="63"/>
+      <c r="AA6" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB6" s="61"/>
+      <c r="AC6" s="62"/>
+      <c r="AD6" s="64"/>
+      <c r="AE6" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="55"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="54" t="s">
-        <v>2</v>
-      </c>
-      <c r="L6" s="55"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="75"/>
-      <c r="O6" s="54" t="s">
-        <v>3</v>
-      </c>
-      <c r="P6" s="55"/>
-      <c r="Q6" s="56"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="54" t="s">
-        <v>4</v>
-      </c>
-      <c r="T6" s="55"/>
-      <c r="U6" s="56"/>
-      <c r="V6" s="56"/>
-      <c r="W6" s="54" t="s">
+      <c r="AF6" s="61"/>
+      <c r="AG6" s="62"/>
+      <c r="AH6" s="62"/>
+      <c r="AI6" s="60" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ6" s="61"/>
+      <c r="AK6" s="62"/>
+      <c r="AL6" s="62"/>
+      <c r="AM6" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="X6" s="55"/>
-      <c r="Y6" s="56"/>
-      <c r="Z6" s="75"/>
-      <c r="AA6" s="54" t="s">
-        <v>5</v>
-      </c>
-      <c r="AB6" s="55"/>
-      <c r="AC6" s="56"/>
-      <c r="AD6" s="57"/>
-      <c r="AE6" s="54" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF6" s="55"/>
-      <c r="AG6" s="56"/>
-      <c r="AH6" s="56"/>
-      <c r="AI6" s="54" t="s">
+      <c r="AN6" s="61"/>
+      <c r="AO6" s="62"/>
+      <c r="AP6" s="63"/>
+      <c r="AQ6" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="AR6" s="61"/>
+      <c r="AS6" s="62"/>
+      <c r="AT6" s="64"/>
+      <c r="AU6" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="AV6" s="66"/>
+      <c r="AW6" s="67"/>
+      <c r="AX6" s="68"/>
+      <c r="AY6" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="73" t="s">
+        <v>1</v>
+      </c>
+      <c r="BA6" s="81" t="s">
+        <v>35</v>
+      </c>
+      <c r="BB6" s="79"/>
+      <c r="BC6" s="79"/>
+      <c r="BD6" s="79"/>
+      <c r="BE6" s="81" t="s">
+        <v>36</v>
+      </c>
+      <c r="BF6" s="79"/>
+      <c r="BG6" s="79"/>
+      <c r="BH6" s="79"/>
+      <c r="BI6" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="BJ6" s="61"/>
+      <c r="BK6" s="62"/>
+      <c r="BL6" s="64"/>
+      <c r="BM6" s="81" t="s">
+        <v>38</v>
+      </c>
+      <c r="BN6" s="79"/>
+      <c r="BO6" s="79"/>
+      <c r="BP6" s="79"/>
+      <c r="BQ6" s="81" t="s">
+        <v>37</v>
+      </c>
+      <c r="BR6" s="79"/>
+      <c r="BS6" s="79"/>
+      <c r="BT6" s="82"/>
+      <c r="BU6" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="BV6" s="79"/>
+      <c r="BW6" s="79"/>
+      <c r="BX6" s="79"/>
+      <c r="BY6" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="AJ6" s="55"/>
-      <c r="AK6" s="56"/>
-      <c r="AL6" s="56"/>
-      <c r="AM6" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="AN6" s="55"/>
-      <c r="AO6" s="56"/>
-      <c r="AP6" s="75"/>
-      <c r="AQ6" s="54" t="s">
-        <v>7</v>
-      </c>
-      <c r="AR6" s="55"/>
-      <c r="AS6" s="56"/>
-      <c r="AT6" s="57"/>
-      <c r="AU6" s="76" t="s">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="77"/>
-      <c r="AW6" s="78"/>
-      <c r="AX6" s="79"/>
-      <c r="AY6" s="66" t="s">
-        <v>0</v>
-      </c>
-      <c r="AZ6" s="68" t="s">
-        <v>1</v>
-      </c>
-      <c r="BA6" s="60" t="s">
-        <v>17</v>
-      </c>
-      <c r="BB6" s="53"/>
-      <c r="BC6" s="53"/>
-      <c r="BD6" s="53"/>
-      <c r="BE6" s="60" t="s">
-        <v>10</v>
-      </c>
-      <c r="BF6" s="53"/>
-      <c r="BG6" s="53"/>
-      <c r="BH6" s="53"/>
-      <c r="BI6" s="54" t="s">
-        <v>18</v>
-      </c>
-      <c r="BJ6" s="55"/>
-      <c r="BK6" s="56"/>
-      <c r="BL6" s="57"/>
-      <c r="BM6" s="60" t="s">
-        <v>6</v>
-      </c>
-      <c r="BN6" s="53"/>
-      <c r="BO6" s="53"/>
-      <c r="BP6" s="53"/>
-      <c r="BQ6" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="BR6" s="53"/>
-      <c r="BS6" s="53"/>
-      <c r="BT6" s="61"/>
-      <c r="BU6" s="53" t="s">
-        <v>34</v>
-      </c>
-      <c r="BV6" s="53"/>
-      <c r="BW6" s="53"/>
-      <c r="BX6" s="53"/>
-      <c r="BY6" s="54" t="s">
-        <v>6</v>
-      </c>
-      <c r="BZ6" s="55"/>
-      <c r="CA6" s="56"/>
-      <c r="CB6" s="57"/>
+      <c r="BZ6" s="61"/>
+      <c r="CA6" s="62"/>
+      <c r="CB6" s="64"/>
     </row>
     <row r="7" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A7" s="67"/>
-      <c r="B7" s="69"/>
+      <c r="A7" s="72"/>
+      <c r="B7" s="74"/>
       <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="F7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="G7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="V7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="X7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AB7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AD7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AE7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AF7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AG7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AH7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="AI7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AJ7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AK7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AL7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="AM7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AN7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AO7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AP7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="AQ7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AR7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AS7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AT7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AU7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="AV7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="AW7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="AX7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="AY7" s="72"/>
+      <c r="AZ7" s="74"/>
+      <c r="BA7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="BB7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="BC7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="BD7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="K7" s="2" t="s">
+      <c r="BE7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="BF7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="BG7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="BH7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="M7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="O7" s="2" t="s">
+      <c r="BI7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="BJ7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="BK7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="P7" s="3" t="s">
+      <c r="BL7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="Q7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="S7" s="2" t="s">
+      <c r="BM7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="BN7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="BO7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="3" t="s">
+      <c r="BP7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="U7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="2" t="s">
+      <c r="BQ7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="BR7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="BS7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="X7" s="3" t="s">
+      <c r="BT7" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="Y7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="2" t="s">
+      <c r="BU7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="BV7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="BW7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AB7" s="3" t="s">
+      <c r="BX7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AC7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE7" s="2" t="s">
+      <c r="BY7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="BZ7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="CA7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AF7" s="3" t="s">
+      <c r="CB7" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="AG7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AH7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AI7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AJ7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AK7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AL7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AM7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AN7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AO7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AP7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="AQ7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AR7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AS7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AT7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AU7" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="AV7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="AW7" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="AX7" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="AY7" s="67"/>
-      <c r="AZ7" s="69"/>
-      <c r="BA7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="BB7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="BC7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="BD7" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="BE7" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="BF7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="BG7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="BH7" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="BI7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="BJ7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="BK7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="BL7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="BM7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="BN7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="BO7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="BP7" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="BQ7" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="BR7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="BS7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="BT7" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="BU7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="BV7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="BW7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="BX7" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="BY7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="BZ7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="CA7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="CB7" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:80" x14ac:dyDescent="0.25">
@@ -7601,10 +7604,10 @@
       </c>
     </row>
     <row r="38" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A38" s="70" t="s">
-        <v>11</v>
-      </c>
-      <c r="B38" s="71"/>
+      <c r="A38" s="75" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" s="76"/>
       <c r="C38" s="33" t="str">
         <f t="shared" ref="C38:AX38" si="29">IF(SUM(C8:C37)=0,"",AVERAGE(C8:C37))</f>
         <v/>
@@ -7797,10 +7800,10 @@
         <f t="shared" si="29"/>
         <v/>
       </c>
-      <c r="AY38" s="70" t="s">
-        <v>11</v>
-      </c>
-      <c r="AZ38" s="71"/>
+      <c r="AY38" s="75" t="s">
+        <v>10</v>
+      </c>
+      <c r="AZ38" s="76"/>
       <c r="BA38" s="33" t="str">
         <f t="shared" ref="BA38:BL38" si="30">IF(SUM(BA8:BA37)=0,"",AVERAGE(BA8:BA37))</f>
         <v/>
@@ -7915,10 +7918,10 @@
       </c>
     </row>
     <row r="39" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A39" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="63"/>
+      <c r="A39" s="77" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" s="78"/>
       <c r="C39" s="33" t="str">
         <f t="shared" ref="C39:AX39" si="33">IF(SUM(C8:C37)=0,"",MEDIAN(C8:C37))</f>
         <v/>
@@ -8111,10 +8114,10 @@
         <f t="shared" si="33"/>
         <v/>
       </c>
-      <c r="AY39" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="AZ39" s="63"/>
+      <c r="AY39" s="77" t="s">
+        <v>11</v>
+      </c>
+      <c r="AZ39" s="78"/>
       <c r="BA39" s="33" t="str">
         <f t="shared" ref="BA39:BL39" si="34">IF(SUM(BA8:BA37)=0,"",MEDIAN(BA8:BA37))</f>
         <v/>
@@ -8229,10 +8232,10 @@
       </c>
     </row>
     <row r="40" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A40" s="62" t="s">
-        <v>13</v>
-      </c>
-      <c r="B40" s="63"/>
+      <c r="A40" s="77" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" s="78"/>
       <c r="C40" s="33" t="str">
         <f t="shared" ref="C40:AX40" si="37">IF(SUM(C8:C37)=0,"",MAX(C8:C37))</f>
         <v/>
@@ -8425,10 +8428,10 @@
         <f t="shared" si="37"/>
         <v/>
       </c>
-      <c r="AY40" s="62" t="s">
-        <v>13</v>
-      </c>
-      <c r="AZ40" s="63"/>
+      <c r="AY40" s="77" t="s">
+        <v>12</v>
+      </c>
+      <c r="AZ40" s="78"/>
       <c r="BA40" s="33" t="str">
         <f t="shared" ref="BA40:BL40" si="38">IF(SUM(BA8:BA37)=0,"",MAX(BA8:BA37))</f>
         <v/>
@@ -8543,10 +8546,10 @@
       </c>
     </row>
     <row r="41" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A41" s="62" t="s">
-        <v>14</v>
-      </c>
-      <c r="B41" s="63"/>
+      <c r="A41" s="77" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="78"/>
       <c r="C41" s="33" t="str">
         <f t="shared" ref="C41:AX41" si="41">IF(SUM(C8:C37)=0,"",MIN(C8:C37))</f>
         <v/>
@@ -8739,10 +8742,10 @@
         <f t="shared" si="41"/>
         <v/>
       </c>
-      <c r="AY41" s="62" t="s">
-        <v>14</v>
-      </c>
-      <c r="AZ41" s="63"/>
+      <c r="AY41" s="77" t="s">
+        <v>13</v>
+      </c>
+      <c r="AZ41" s="78"/>
       <c r="BA41" s="33" t="str">
         <f t="shared" ref="BA41:BL41" si="42">IF(SUM(BA8:BA37)=0,"",MIN(BA8:BA37))</f>
         <v/>
@@ -8857,10 +8860,10 @@
       </c>
     </row>
     <row r="42" spans="1:80" x14ac:dyDescent="0.25">
-      <c r="A42" s="64" t="s">
-        <v>15</v>
-      </c>
-      <c r="B42" s="65"/>
+      <c r="A42" s="69" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="70"/>
       <c r="C42" s="2" t="str">
         <f t="shared" ref="C42:AX42" si="45">IF(C38="","",COUNTIF(C8:C37,"&lt;51")/COUNT(C8:C37)*100)</f>
         <v/>
@@ -9053,10 +9056,10 @@
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="AY42" s="64" t="s">
-        <v>15</v>
-      </c>
-      <c r="AZ42" s="65"/>
+      <c r="AY42" s="69" t="s">
+        <v>14</v>
+      </c>
+      <c r="AZ42" s="70"/>
       <c r="BA42" s="2" t="str">
         <f t="shared" ref="BA42:BL42" si="46">IF(BA38="","",COUNTIF(BA8:BA37,"&lt;51")/COUNT(BA8:BA37)*100)</f>
         <v/>
@@ -9476,175 +9479,196 @@
     </row>
     <row r="50" spans="1:79" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="51" spans="1:79" x14ac:dyDescent="0.25">
-      <c r="B51" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="C51" s="80"/>
-      <c r="D51" s="80"/>
-      <c r="E51" s="80"/>
-      <c r="F51" s="80"/>
-      <c r="G51" s="80"/>
+      <c r="B51" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="C51" s="55"/>
+      <c r="D51" s="55"/>
+      <c r="E51" s="55"/>
+      <c r="F51" s="55"/>
+      <c r="G51" s="55"/>
       <c r="H51" s="52"/>
       <c r="I51" s="52"/>
       <c r="J51" s="52"/>
-      <c r="M51" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="N51" s="80"/>
-      <c r="O51" s="80"/>
-      <c r="P51" s="80"/>
-      <c r="Q51" s="80"/>
-      <c r="R51" s="80"/>
-      <c r="S51" s="80"/>
-      <c r="T51" s="80"/>
-      <c r="U51" s="80"/>
-      <c r="V51" s="80"/>
-      <c r="W51" s="80"/>
-      <c r="X51" s="80"/>
+      <c r="M51" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="N51" s="55"/>
+      <c r="O51" s="55"/>
+      <c r="P51" s="55"/>
+      <c r="Q51" s="55"/>
+      <c r="R51" s="55"/>
+      <c r="S51" s="55"/>
+      <c r="T51" s="55"/>
+      <c r="U51" s="55"/>
+      <c r="V51" s="55"/>
+      <c r="W51" s="55"/>
+      <c r="X51" s="55"/>
       <c r="Y51" s="52"/>
       <c r="Z51" s="52"/>
-      <c r="AD51" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="AE51" s="80"/>
-      <c r="AF51" s="80"/>
-      <c r="AG51" s="80"/>
-      <c r="AH51" s="80"/>
-      <c r="AI51" s="80"/>
-      <c r="AJ51" s="80"/>
-      <c r="AK51" s="80"/>
-      <c r="AL51" s="80"/>
-      <c r="AM51" s="80"/>
-      <c r="AN51" s="80"/>
-      <c r="AO51" s="80"/>
+      <c r="AD51" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="AE51" s="55"/>
+      <c r="AF51" s="55"/>
+      <c r="AG51" s="55"/>
+      <c r="AH51" s="55"/>
+      <c r="AI51" s="55"/>
+      <c r="AJ51" s="55"/>
+      <c r="AK51" s="55"/>
+      <c r="AL51" s="55"/>
+      <c r="AM51" s="55"/>
+      <c r="AN51" s="55"/>
+      <c r="AO51" s="55"/>
       <c r="AP51" s="52"/>
-      <c r="AY51" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="AZ51" s="80"/>
-      <c r="BA51" s="82"/>
-      <c r="BB51" s="82"/>
-      <c r="BC51" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="BD51" s="80"/>
-      <c r="BE51" s="80"/>
-      <c r="BF51" s="80"/>
-      <c r="BG51" s="80"/>
-      <c r="BH51" s="80"/>
-      <c r="BI51" s="80"/>
-      <c r="BJ51" s="80"/>
-      <c r="BK51" s="80"/>
-      <c r="BL51" s="80"/>
-      <c r="BM51" s="80"/>
-      <c r="BN51" s="80"/>
-      <c r="BO51" s="82"/>
-      <c r="BP51" s="80" t="s">
-        <v>22</v>
-      </c>
-      <c r="BQ51" s="80"/>
-      <c r="BR51" s="80"/>
-      <c r="BS51" s="80"/>
-      <c r="BT51" s="80"/>
-      <c r="BU51" s="80"/>
-      <c r="BV51" s="80"/>
-      <c r="BW51" s="80"/>
-      <c r="BX51" s="80"/>
-      <c r="BY51" s="80"/>
+      <c r="AY51" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="AZ51" s="55"/>
+      <c r="BA51" s="53"/>
+      <c r="BB51" s="53"/>
+      <c r="BC51" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="BD51" s="55"/>
+      <c r="BE51" s="55"/>
+      <c r="BF51" s="55"/>
+      <c r="BG51" s="55"/>
+      <c r="BH51" s="55"/>
+      <c r="BI51" s="55"/>
+      <c r="BJ51" s="55"/>
+      <c r="BK51" s="55"/>
+      <c r="BL51" s="55"/>
+      <c r="BM51" s="55"/>
+      <c r="BN51" s="55"/>
+      <c r="BO51" s="53"/>
+      <c r="BP51" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="BQ51" s="55"/>
+      <c r="BR51" s="55"/>
+      <c r="BS51" s="55"/>
+      <c r="BT51" s="55"/>
+      <c r="BU51" s="55"/>
+      <c r="BV51" s="55"/>
+      <c r="BW51" s="55"/>
+      <c r="BX51" s="55"/>
+      <c r="BY51" s="55"/>
     </row>
     <row r="52" spans="1:79" x14ac:dyDescent="0.25">
-      <c r="B52" s="81" t="s">
-        <v>36</v>
-      </c>
-      <c r="C52" s="81"/>
-      <c r="D52" s="81"/>
-      <c r="E52" s="81"/>
-      <c r="F52" s="81"/>
-      <c r="G52" s="81"/>
+      <c r="B52" s="54" t="s">
+        <v>32</v>
+      </c>
+      <c r="C52" s="54"/>
+      <c r="D52" s="54"/>
+      <c r="E52" s="54"/>
+      <c r="F52" s="54"/>
+      <c r="G52" s="54"/>
       <c r="H52" s="52"/>
       <c r="I52" s="52"/>
       <c r="J52" s="52"/>
-      <c r="M52" s="81" t="s">
-        <v>23</v>
-      </c>
-      <c r="N52" s="81"/>
-      <c r="O52" s="81"/>
-      <c r="P52" s="81"/>
-      <c r="Q52" s="81"/>
-      <c r="R52" s="81"/>
-      <c r="S52" s="81"/>
-      <c r="T52" s="81"/>
-      <c r="U52" s="81"/>
-      <c r="V52" s="81"/>
-      <c r="W52" s="81"/>
-      <c r="X52" s="81"/>
+      <c r="M52" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="N52" s="54"/>
+      <c r="O52" s="54"/>
+      <c r="P52" s="54"/>
+      <c r="Q52" s="54"/>
+      <c r="R52" s="54"/>
+      <c r="S52" s="54"/>
+      <c r="T52" s="54"/>
+      <c r="U52" s="54"/>
+      <c r="V52" s="54"/>
+      <c r="W52" s="54"/>
+      <c r="X52" s="54"/>
       <c r="Y52" s="52"/>
       <c r="Z52" s="52"/>
-      <c r="AD52" s="81" t="s">
-        <v>24</v>
-      </c>
-      <c r="AE52" s="81"/>
-      <c r="AF52" s="81"/>
-      <c r="AG52" s="81"/>
-      <c r="AH52" s="81"/>
-      <c r="AI52" s="81"/>
-      <c r="AJ52" s="81"/>
-      <c r="AK52" s="81"/>
-      <c r="AL52" s="81"/>
-      <c r="AM52" s="81"/>
-      <c r="AN52" s="81"/>
-      <c r="AO52" s="81"/>
+      <c r="AD52" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE52" s="54"/>
+      <c r="AF52" s="54"/>
+      <c r="AG52" s="54"/>
+      <c r="AH52" s="54"/>
+      <c r="AI52" s="54"/>
+      <c r="AJ52" s="54"/>
+      <c r="AK52" s="54"/>
+      <c r="AL52" s="54"/>
+      <c r="AM52" s="54"/>
+      <c r="AN52" s="54"/>
+      <c r="AO52" s="54"/>
       <c r="AP52" s="52"/>
       <c r="AW52" t="s">
-        <v>37</v>
-      </c>
-      <c r="AY52" s="81" t="s">
-        <v>36</v>
-      </c>
-      <c r="AZ52" s="81"/>
+        <v>33</v>
+      </c>
+      <c r="AY52" s="54" t="s">
+        <v>32</v>
+      </c>
+      <c r="AZ52" s="54"/>
       <c r="BA52" s="52"/>
       <c r="BB52" s="52"/>
-      <c r="BC52" s="81" t="s">
-        <v>23</v>
-      </c>
-      <c r="BD52" s="81"/>
-      <c r="BE52" s="81"/>
-      <c r="BF52" s="81"/>
-      <c r="BG52" s="81"/>
-      <c r="BH52" s="81"/>
-      <c r="BI52" s="81"/>
-      <c r="BJ52" s="81"/>
-      <c r="BK52" s="81"/>
-      <c r="BL52" s="81"/>
-      <c r="BM52" s="81"/>
-      <c r="BN52" s="81"/>
+      <c r="BC52" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="BD52" s="54"/>
+      <c r="BE52" s="54"/>
+      <c r="BF52" s="54"/>
+      <c r="BG52" s="54"/>
+      <c r="BH52" s="54"/>
+      <c r="BI52" s="54"/>
+      <c r="BJ52" s="54"/>
+      <c r="BK52" s="54"/>
+      <c r="BL52" s="54"/>
+      <c r="BM52" s="54"/>
+      <c r="BN52" s="54"/>
       <c r="BO52" s="52"/>
-      <c r="BP52" s="81" t="s">
-        <v>24</v>
-      </c>
-      <c r="BQ52" s="81"/>
-      <c r="BR52" s="81"/>
-      <c r="BS52" s="81"/>
-      <c r="BT52" s="81"/>
-      <c r="BU52" s="81"/>
-      <c r="BV52" s="81"/>
-      <c r="BW52" s="81"/>
-      <c r="BX52" s="81"/>
-      <c r="BY52" s="81"/>
+      <c r="BP52" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="BQ52" s="54"/>
+      <c r="BR52" s="54"/>
+      <c r="BS52" s="54"/>
+      <c r="BT52" s="54"/>
+      <c r="BU52" s="54"/>
+      <c r="BV52" s="54"/>
+      <c r="BW52" s="54"/>
+      <c r="BX52" s="54"/>
+      <c r="BY52" s="54"/>
       <c r="CA52" s="51" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B52:G52"/>
-    <mergeCell ref="M52:X52"/>
-    <mergeCell ref="AD52:AO52"/>
-    <mergeCell ref="AY51:AZ51"/>
-    <mergeCell ref="B51:G51"/>
-    <mergeCell ref="M51:X51"/>
-    <mergeCell ref="AD51:AO51"/>
-    <mergeCell ref="AY52:AZ52"/>
+    <mergeCell ref="BU6:BX6"/>
+    <mergeCell ref="BY6:CB6"/>
+    <mergeCell ref="AY2:CB2"/>
+    <mergeCell ref="AY3:CB3"/>
+    <mergeCell ref="AY4:CB4"/>
+    <mergeCell ref="AY5:CB5"/>
+    <mergeCell ref="BA6:BD6"/>
+    <mergeCell ref="BE6:BH6"/>
+    <mergeCell ref="BI6:BL6"/>
+    <mergeCell ref="BM6:BP6"/>
+    <mergeCell ref="BQ6:BT6"/>
+    <mergeCell ref="AY41:AZ41"/>
+    <mergeCell ref="AY42:AZ42"/>
+    <mergeCell ref="AY6:AY7"/>
+    <mergeCell ref="AZ6:AZ7"/>
+    <mergeCell ref="AY38:AZ38"/>
+    <mergeCell ref="AY39:AZ39"/>
+    <mergeCell ref="AY40:AZ40"/>
+    <mergeCell ref="AA6:AD6"/>
+    <mergeCell ref="AE6:AH6"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
     <mergeCell ref="BP51:BY51"/>
     <mergeCell ref="BP52:BY52"/>
     <mergeCell ref="BC51:BN51"/>
@@ -9661,35 +9685,14 @@
     <mergeCell ref="S6:V6"/>
     <mergeCell ref="W6:Z6"/>
     <mergeCell ref="AI6:AL6"/>
-    <mergeCell ref="AA6:AD6"/>
-    <mergeCell ref="AE6:AH6"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="AY41:AZ41"/>
-    <mergeCell ref="AY42:AZ42"/>
-    <mergeCell ref="AY6:AY7"/>
-    <mergeCell ref="AZ6:AZ7"/>
-    <mergeCell ref="AY38:AZ38"/>
-    <mergeCell ref="AY39:AZ39"/>
-    <mergeCell ref="AY40:AZ40"/>
-    <mergeCell ref="BU6:BX6"/>
-    <mergeCell ref="BY6:CB6"/>
-    <mergeCell ref="AY2:CB2"/>
-    <mergeCell ref="AY3:CB3"/>
-    <mergeCell ref="AY4:CB4"/>
-    <mergeCell ref="AY5:CB5"/>
-    <mergeCell ref="BA6:BD6"/>
-    <mergeCell ref="BE6:BH6"/>
-    <mergeCell ref="BI6:BL6"/>
-    <mergeCell ref="BM6:BP6"/>
-    <mergeCell ref="BQ6:BT6"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="M52:X52"/>
+    <mergeCell ref="AD52:AO52"/>
+    <mergeCell ref="AY51:AZ51"/>
+    <mergeCell ref="B51:G51"/>
+    <mergeCell ref="M51:X51"/>
+    <mergeCell ref="AD51:AO51"/>
+    <mergeCell ref="AY52:AZ52"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:AX37 BA8:BL37">
     <cfRule type="cellIs" dxfId="3" priority="5" operator="between">

</xml_diff>